<commit_message>
docs: propuesta de base de datos v2 (ficha 19, diagrama 8) y HU-19 en el backlog
</commit_message>
<xml_diff>
--- a/docs/fase2/evidencias_proyecto/documentacion/agil/product_backlog.xlsx
+++ b/docs/fase2/evidencias_proyecto/documentacion/agil/product_backlog.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Resumen" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Product Backlog'!$A$4:$I$22</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Product Backlog'!$A$4:$I$23</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="119">
   <si>
     <t xml:space="preserve">DomoVida · Product Backlog priorizado (actualizado al 6 de octubre de 2026)</t>
   </si>
@@ -357,6 +357,21 @@
   </si>
   <si>
     <t xml:space="preserve">Sin capacidad gratuita en la región (03 y 05/10).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HU-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como personal técnico, quiero rediseñar la base de datos (modelo v2), para sincronizar el modo borde sin duplicados, aplicar RLS por cuidador y mantener una sola fuente de verdad de las alertas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dado el modelo v2 migrado con migraciones versionadas, cuando se reconstruye la base desde el repositorio y se repiten PR-03 y PS-01b, entonces no hay eventos duplicados, cada fecha tiene zona horaria y la atención queda registrada en alertas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PI-06, PR-03, PS-03 (por definir)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agregada el 06/10. Diagnóstico y plan en la ficha técnica 19 y el diagrama 08.</t>
   </si>
   <si>
     <t xml:space="preserve">Resumen del backlog</t>
@@ -921,7 +936,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -1494,8 +1509,37 @@
         <v>110</v>
       </c>
     </row>
+    <row r="23" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="G23" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="H23" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="I23" s="5" t="s">
+        <v>115</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I22"/>
+  <autoFilter ref="A4:I23"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
@@ -1525,7 +1569,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1533,7 +1577,7 @@
         <v>8</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="C3" s="11" t="s">
         <v>13</v>
@@ -1550,19 +1594,19 @@
         <v>17</v>
       </c>
       <c r="B4" s="12" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$22,A4)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$23,A4)</f>
         <v>14</v>
       </c>
       <c r="C4" s="12" t="n">
-        <f aca="false">COUNTIFS('Product Backlog'!$G$5:$G$22,$A4,'Product Backlog'!$C$5:$C$22,"Must")</f>
+        <f aca="false">COUNTIFS('Product Backlog'!$G$5:$G$23,$A4,'Product Backlog'!$C$5:$C$23,"Must")</f>
         <v>9</v>
       </c>
       <c r="D4" s="12" t="n">
-        <f aca="false">COUNTIFS('Product Backlog'!$G$5:$G$22,$A4,'Product Backlog'!$C$5:$C$22,"Should")</f>
+        <f aca="false">COUNTIFS('Product Backlog'!$G$5:$G$23,$A4,'Product Backlog'!$C$5:$C$23,"Should")</f>
         <v>4</v>
       </c>
       <c r="E4" s="12" t="n">
-        <f aca="false">COUNTIFS('Product Backlog'!$G$5:$G$22,$A4,'Product Backlog'!$C$5:$C$22,"Could")</f>
+        <f aca="false">COUNTIFS('Product Backlog'!$G$5:$G$23,$A4,'Product Backlog'!$C$5:$C$23,"Could")</f>
         <v>1</v>
       </c>
     </row>
@@ -1571,19 +1615,19 @@
         <v>31</v>
       </c>
       <c r="B5" s="12" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$22,A5)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$23,A5)</f>
         <v>1</v>
       </c>
       <c r="C5" s="12" t="n">
-        <f aca="false">COUNTIFS('Product Backlog'!$G$5:$G$22,$A5,'Product Backlog'!$C$5:$C$22,"Must")</f>
+        <f aca="false">COUNTIFS('Product Backlog'!$G$5:$G$23,$A5,'Product Backlog'!$C$5:$C$23,"Must")</f>
         <v>1</v>
       </c>
       <c r="D5" s="12" t="n">
-        <f aca="false">COUNTIFS('Product Backlog'!$G$5:$G$22,$A5,'Product Backlog'!$C$5:$C$22,"Should")</f>
+        <f aca="false">COUNTIFS('Product Backlog'!$G$5:$G$23,$A5,'Product Backlog'!$C$5:$C$23,"Should")</f>
         <v>0</v>
       </c>
       <c r="E5" s="12" t="n">
-        <f aca="false">COUNTIFS('Product Backlog'!$G$5:$G$22,$A5,'Product Backlog'!$C$5:$C$22,"Could")</f>
+        <f aca="false">COUNTIFS('Product Backlog'!$G$5:$G$23,$A5,'Product Backlog'!$C$5:$C$23,"Could")</f>
         <v>0</v>
       </c>
     </row>
@@ -1592,19 +1636,19 @@
         <v>79</v>
       </c>
       <c r="B6" s="12" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$22,A6)</f>
-        <v>2</v>
+        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$23,A6)</f>
+        <v>3</v>
       </c>
       <c r="C6" s="12" t="n">
-        <f aca="false">COUNTIFS('Product Backlog'!$G$5:$G$22,$A6,'Product Backlog'!$C$5:$C$22,"Must")</f>
+        <f aca="false">COUNTIFS('Product Backlog'!$G$5:$G$23,$A6,'Product Backlog'!$C$5:$C$23,"Must")</f>
         <v>0</v>
       </c>
       <c r="D6" s="12" t="n">
-        <f aca="false">COUNTIFS('Product Backlog'!$G$5:$G$22,$A6,'Product Backlog'!$C$5:$C$22,"Should")</f>
-        <v>2</v>
+        <f aca="false">COUNTIFS('Product Backlog'!$G$5:$G$23,$A6,'Product Backlog'!$C$5:$C$23,"Should")</f>
+        <v>3</v>
       </c>
       <c r="E6" s="12" t="n">
-        <f aca="false">COUNTIFS('Product Backlog'!$G$5:$G$22,$A6,'Product Backlog'!$C$5:$C$22,"Could")</f>
+        <f aca="false">COUNTIFS('Product Backlog'!$G$5:$G$23,$A6,'Product Backlog'!$C$5:$C$23,"Could")</f>
         <v>0</v>
       </c>
     </row>
@@ -1613,29 +1657,29 @@
         <v>108</v>
       </c>
       <c r="B7" s="12" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$22,A7)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$G$5:$G$23,A7)</f>
         <v>1</v>
       </c>
       <c r="C7" s="12" t="n">
-        <f aca="false">COUNTIFS('Product Backlog'!$G$5:$G$22,$A7,'Product Backlog'!$C$5:$C$22,"Must")</f>
+        <f aca="false">COUNTIFS('Product Backlog'!$G$5:$G$23,$A7,'Product Backlog'!$C$5:$C$23,"Must")</f>
         <v>0</v>
       </c>
       <c r="D7" s="12" t="n">
-        <f aca="false">COUNTIFS('Product Backlog'!$G$5:$G$22,$A7,'Product Backlog'!$C$5:$C$22,"Should")</f>
+        <f aca="false">COUNTIFS('Product Backlog'!$G$5:$G$23,$A7,'Product Backlog'!$C$5:$C$23,"Should")</f>
         <v>0</v>
       </c>
       <c r="E7" s="12" t="n">
-        <f aca="false">COUNTIFS('Product Backlog'!$G$5:$G$22,$A7,'Product Backlog'!$C$5:$C$22,"Could")</f>
+        <f aca="false">COUNTIFS('Product Backlog'!$G$5:$G$23,$A7,'Product Backlog'!$C$5:$C$23,"Could")</f>
         <v>1</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="B8" s="13" t="n">
         <f aca="false">SUM(B4:B7)</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C8" s="13" t="n">
         <f aca="false">SUM(C4:C7)</f>
@@ -1643,7 +1687,7 @@
       </c>
       <c r="D8" s="13" t="n">
         <f aca="false">SUM(D4:D7)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E8" s="13" t="n">
         <f aca="false">SUM(E4:E7)</f>

</xml_diff>